<commit_message>
adds new redd data, updated csvs
</commit_message>
<xml_diff>
--- a/data-raw/metadata/clear_redd_summary_metadata.xlsx
+++ b/data-raw/metadata/clear_redd_summary_metadata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Badhia\Documents\git\jpe-clear-adult-edi\data-raw\metadata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73A262B8-FCAD-4B29-9455-23D4AB58F84B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2FA72F7-9A2F-4EC1-8E42-99736B439489}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1990" yWindow="2140" windowWidth="19200" windowHeight="11180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6740" yWindow="1120" windowWidth="17720" windowHeight="13260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="attribute" sheetId="1" r:id="rId1"/>
@@ -94,9 +94,6 @@
     <t>Total annual count of unique redds. Redd surveys are conducted as repeat observations where a given redd may be recorded multiple times. This field counts only unique redds.</t>
   </si>
   <si>
-    <t>5</t>
-  </si>
-  <si>
     <t>number_reaches_surveyed</t>
   </si>
   <si>
@@ -121,12 +118,6 @@
     <t>149</t>
   </si>
   <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
     <t>2024</t>
   </si>
   <si>
@@ -140,6 +131,15 @@
   </si>
   <si>
     <t>text</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>5.5</t>
+  </si>
+  <si>
+    <t>7</t>
   </si>
 </sst>
 </file>
@@ -547,7 +547,7 @@
         <v>13</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E2" s="13" t="s">
         <v>14</v>
@@ -559,16 +559,16 @@
         <v>18</v>
       </c>
       <c r="H2" s="15" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I2" s="14"/>
       <c r="J2" s="15"/>
       <c r="K2" s="14"/>
       <c r="L2" s="16" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="M2" s="16" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="N2" s="7"/>
       <c r="O2" s="7"/>
@@ -595,7 +595,7 @@
         <v>13</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E3" s="13" t="s">
         <v>14</v>
@@ -604,19 +604,19 @@
         <v>13</v>
       </c>
       <c r="G3" s="15" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H3" s="15" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I3" s="14"/>
       <c r="J3" s="15"/>
       <c r="K3" s="14"/>
       <c r="L3" s="16" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="M3" s="16" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N3" s="7"/>
       <c r="O3" s="7"/>
@@ -634,16 +634,16 @@
     </row>
     <row r="4" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A4" s="13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C4" s="13" t="s">
         <v>13</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E4" s="13" t="s">
         <v>14</v>
@@ -652,19 +652,19 @@
         <v>13</v>
       </c>
       <c r="G4" s="15" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H4" s="15" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I4" s="14"/>
       <c r="J4" s="15"/>
       <c r="K4" s="14"/>
       <c r="L4" s="16" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="M4" s="16" t="s">
-        <v>22</v>
+        <v>37</v>
       </c>
       <c r="N4" s="7"/>
       <c r="O4" s="7"/>
@@ -682,19 +682,19 @@
     </row>
     <row r="5" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" s="4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>

</xml_diff>

<commit_message>
adds survey days total to redd summary, updates metadata
</commit_message>
<xml_diff>
--- a/data-raw/metadata/clear_redd_summary_metadata.xlsx
+++ b/data-raw/metadata/clear_redd_summary_metadata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Badhia\Documents\git\jpe-clear-adult-edi\data-raw\metadata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2FA72F7-9A2F-4EC1-8E42-99736B439489}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D25CFD2-529D-4927-933F-43FCE5A0F36F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6740" yWindow="1120" windowWidth="17720" windowHeight="13260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-27735" yWindow="2835" windowWidth="16530" windowHeight="11205" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="attribute" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="41">
   <si>
     <t xml:space="preserve">attribute_name </t>
   </si>
@@ -141,12 +141,21 @@
   <si>
     <t>7</t>
   </si>
+  <si>
+    <t>total_number_of_survey_days</t>
+  </si>
+  <si>
+    <t>Total survey days that year</t>
+  </si>
+  <si>
+    <t>day</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
@@ -187,6 +196,12 @@
       <color rgb="FF000000"/>
       <name val="Aptos"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -220,7 +235,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -248,6 +263,8 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="49" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -719,19 +736,39 @@
       <c r="Z5" s="7"/>
     </row>
     <row r="6" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="4"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="6"/>
-      <c r="G6" s="6"/>
-      <c r="H6" s="6"/>
+      <c r="A6" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G6" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>24</v>
+      </c>
       <c r="I6" s="5"/>
       <c r="J6" s="6"/>
       <c r="K6" s="5"/>
-      <c r="L6" s="10"/>
-      <c r="M6" s="10"/>
+      <c r="L6" s="10">
+        <v>10</v>
+      </c>
+      <c r="M6" s="10">
+        <v>76</v>
+      </c>
       <c r="N6" s="7"/>
       <c r="O6" s="7"/>
       <c r="P6" s="7"/>

</xml_diff>

<commit_message>
removes total surveyed days from redd summary, adds environmentals file
</commit_message>
<xml_diff>
--- a/data-raw/metadata/clear_redd_summary_metadata.xlsx
+++ b/data-raw/metadata/clear_redd_summary_metadata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Badhia\Documents\git\jpe-clear-adult-edi\data-raw\metadata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{631E368E-2F03-46B4-ACBB-FBDDAEE4E454}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B91AFB5-A8EA-42CE-8437-5945C64FE1A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8140" yWindow="2210" windowWidth="14500" windowHeight="10460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5650" yWindow="2160" windowWidth="19200" windowHeight="11170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="attribute" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="38">
   <si>
     <t xml:space="preserve">attribute_name </t>
   </si>
@@ -136,15 +136,6 @@
     <t>7</t>
   </si>
   <si>
-    <t>total_number_of_survey_days</t>
-  </si>
-  <si>
-    <t>Total survey days that year</t>
-  </si>
-  <si>
-    <t>day</t>
-  </si>
-  <si>
     <t>reaches_numbers</t>
   </si>
   <si>
@@ -155,7 +146,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
@@ -196,12 +187,6 @@
       <color rgb="FF000000"/>
       <name val="Aptos"/>
     </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -235,7 +220,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -263,8 +248,6 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="49" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -480,7 +463,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z992"/>
+  <dimension ref="A1:Z991"/>
   <sheetFormatPr defaultColWidth="11.1640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="16.33203125" style="8" bestFit="1" customWidth="1"/>
@@ -699,10 +682,10 @@
     </row>
     <row r="5" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>31</v>
@@ -736,39 +719,19 @@
       <c r="Z5" s="7"/>
     </row>
     <row r="6" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="17" t="s">
-        <v>36</v>
-      </c>
-      <c r="B6" s="17" t="s">
-        <v>37</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D6" s="14" t="s">
-        <v>25</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="G6" s="18" t="s">
-        <v>38</v>
-      </c>
-      <c r="H6" s="6" t="s">
-        <v>24</v>
-      </c>
+      <c r="A6" s="4"/>
+      <c r="B6" s="4"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="6"/>
+      <c r="G6" s="6"/>
+      <c r="H6" s="6"/>
       <c r="I6" s="5"/>
       <c r="J6" s="6"/>
       <c r="K6" s="5"/>
-      <c r="L6" s="10">
-        <v>10</v>
-      </c>
-      <c r="M6" s="10">
-        <v>76</v>
-      </c>
+      <c r="L6" s="10"/>
+      <c r="M6" s="6"/>
       <c r="N6" s="7"/>
       <c r="O6" s="7"/>
       <c r="P6" s="7"/>
@@ -823,7 +786,7 @@
       <c r="I8" s="5"/>
       <c r="J8" s="6"/>
       <c r="K8" s="5"/>
-      <c r="L8" s="10"/>
+      <c r="L8" s="9"/>
       <c r="M8" s="6"/>
       <c r="N8" s="7"/>
       <c r="O8" s="7"/>
@@ -841,18 +804,18 @@
     </row>
     <row r="9" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A9" s="4"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="4"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="6"/>
-      <c r="G9" s="6"/>
-      <c r="H9" s="6"/>
-      <c r="I9" s="5"/>
-      <c r="J9" s="6"/>
-      <c r="K9" s="5"/>
-      <c r="L9" s="9"/>
-      <c r="M9" s="6"/>
+      <c r="B9" s="7"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="12"/>
+      <c r="G9" s="12"/>
+      <c r="H9" s="12"/>
+      <c r="I9" s="11"/>
+      <c r="J9" s="12"/>
+      <c r="K9" s="11"/>
+      <c r="L9" s="12"/>
+      <c r="M9" s="12"/>
       <c r="N9" s="7"/>
       <c r="O9" s="7"/>
       <c r="P9" s="7"/>
@@ -951,9 +914,8 @@
       <c r="Y12" s="7"/>
       <c r="Z12" s="7"/>
     </row>
-    <row r="13" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A13" s="4"/>
-      <c r="B13" s="7"/>
       <c r="C13" s="7"/>
       <c r="D13" s="11"/>
       <c r="E13" s="7"/>
@@ -979,8 +941,9 @@
       <c r="Y13" s="7"/>
       <c r="Z13" s="7"/>
     </row>
-    <row r="14" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A14" s="4"/>
+      <c r="B14" s="7"/>
       <c r="C14" s="7"/>
       <c r="D14" s="11"/>
       <c r="E14" s="7"/>
@@ -1148,34 +1111,34 @@
     </row>
     <row r="20" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A20" s="4"/>
-      <c r="B20" s="7"/>
       <c r="C20" s="7"/>
       <c r="D20" s="11"/>
       <c r="E20" s="7"/>
-      <c r="F20" s="12"/>
-      <c r="G20" s="12"/>
-      <c r="H20" s="12"/>
-      <c r="I20" s="11"/>
-      <c r="J20" s="12"/>
-      <c r="K20" s="11"/>
+      <c r="F20" s="6"/>
+      <c r="G20" s="6"/>
+      <c r="H20" s="6"/>
+      <c r="I20" s="5"/>
+      <c r="J20" s="6"/>
+      <c r="K20" s="5"/>
       <c r="L20" s="12"/>
-      <c r="M20" s="12"/>
-      <c r="N20" s="7"/>
-      <c r="O20" s="7"/>
-      <c r="P20" s="7"/>
-      <c r="Q20" s="7"/>
-      <c r="R20" s="7"/>
-      <c r="S20" s="7"/>
-      <c r="T20" s="7"/>
-      <c r="U20" s="7"/>
-      <c r="V20" s="7"/>
-      <c r="W20" s="7"/>
-      <c r="X20" s="7"/>
-      <c r="Y20" s="7"/>
-      <c r="Z20" s="7"/>
+      <c r="M20" s="6"/>
+      <c r="N20" s="4"/>
+      <c r="O20" s="4"/>
+      <c r="P20" s="4"/>
+      <c r="Q20" s="4"/>
+      <c r="R20" s="4"/>
+      <c r="S20" s="4"/>
+      <c r="T20" s="4"/>
+      <c r="U20" s="4"/>
+      <c r="V20" s="4"/>
+      <c r="W20" s="4"/>
+      <c r="X20" s="4"/>
+      <c r="Y20" s="4"/>
+      <c r="Z20" s="4"/>
     </row>
     <row r="21" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A21" s="4"/>
+      <c r="B21" s="7"/>
       <c r="C21" s="7"/>
       <c r="D21" s="11"/>
       <c r="E21" s="7"/>
@@ -1185,7 +1148,7 @@
       <c r="I21" s="5"/>
       <c r="J21" s="6"/>
       <c r="K21" s="5"/>
-      <c r="L21" s="12"/>
+      <c r="L21" s="6"/>
       <c r="M21" s="6"/>
       <c r="N21" s="4"/>
       <c r="O21" s="4"/>
@@ -1207,39 +1170,29 @@
       <c r="C22" s="7"/>
       <c r="D22" s="11"/>
       <c r="E22" s="7"/>
-      <c r="F22" s="6"/>
-      <c r="G22" s="6"/>
-      <c r="H22" s="6"/>
-      <c r="I22" s="5"/>
-      <c r="J22" s="6"/>
-      <c r="K22" s="5"/>
-      <c r="L22" s="6"/>
-      <c r="M22" s="6"/>
-      <c r="N22" s="4"/>
-      <c r="O22" s="4"/>
-      <c r="P22" s="4"/>
-      <c r="Q22" s="4"/>
-      <c r="R22" s="4"/>
-      <c r="S22" s="4"/>
-      <c r="T22" s="4"/>
-      <c r="U22" s="4"/>
-      <c r="V22" s="4"/>
-      <c r="W22" s="4"/>
-      <c r="X22" s="4"/>
-      <c r="Y22" s="4"/>
-      <c r="Z22" s="4"/>
+      <c r="F22" s="12"/>
+      <c r="G22" s="12"/>
+      <c r="H22" s="12"/>
+      <c r="I22" s="11"/>
+      <c r="J22" s="12"/>
+      <c r="K22" s="11"/>
+      <c r="L22" s="12"/>
+      <c r="M22" s="12"/>
+      <c r="N22" s="7"/>
+      <c r="O22" s="7"/>
+      <c r="P22" s="7"/>
+      <c r="Q22" s="7"/>
+      <c r="R22" s="7"/>
+      <c r="S22" s="7"/>
+      <c r="T22" s="7"/>
+      <c r="U22" s="7"/>
+      <c r="V22" s="7"/>
+      <c r="W22" s="7"/>
+      <c r="X22" s="7"/>
+      <c r="Y22" s="7"/>
+      <c r="Z22" s="7"/>
     </row>
     <row r="23" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A23" s="4"/>
-      <c r="B23" s="7"/>
-      <c r="C23" s="7"/>
-      <c r="D23" s="11"/>
-      <c r="E23" s="7"/>
-      <c r="F23" s="12"/>
-      <c r="G23" s="12"/>
-      <c r="H23" s="12"/>
-      <c r="I23" s="11"/>
-      <c r="J23" s="12"/>
       <c r="K23" s="11"/>
       <c r="L23" s="12"/>
       <c r="M23" s="12"/>
@@ -1258,6 +1211,16 @@
       <c r="Z23" s="7"/>
     </row>
     <row r="24" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A24" s="4"/>
+      <c r="B24" s="7"/>
+      <c r="C24" s="7"/>
+      <c r="D24" s="11"/>
+      <c r="E24" s="7"/>
+      <c r="F24" s="12"/>
+      <c r="G24" s="12"/>
+      <c r="H24" s="12"/>
+      <c r="I24" s="11"/>
+      <c r="J24" s="12"/>
       <c r="K24" s="11"/>
       <c r="L24" s="12"/>
       <c r="M24" s="12"/>
@@ -1388,7 +1351,6 @@
       <c r="Z28" s="7"/>
     </row>
     <row r="29" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A29" s="4"/>
       <c r="B29" s="7"/>
       <c r="C29" s="7"/>
       <c r="D29" s="11"/>
@@ -1416,6 +1378,7 @@
       <c r="Z29" s="7"/>
     </row>
     <row r="30" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A30" s="4"/>
       <c r="B30" s="7"/>
       <c r="C30" s="7"/>
       <c r="D30" s="11"/>
@@ -1443,7 +1406,6 @@
       <c r="Z30" s="7"/>
     </row>
     <row r="31" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A31" s="4"/>
       <c r="B31" s="7"/>
       <c r="C31" s="7"/>
       <c r="D31" s="11"/>
@@ -1471,6 +1433,7 @@
       <c r="Z31" s="7"/>
     </row>
     <row r="32" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A32" s="4"/>
       <c r="B32" s="7"/>
       <c r="C32" s="7"/>
       <c r="D32" s="11"/>
@@ -2422,7 +2385,7 @@
       <c r="Z65" s="7"/>
     </row>
     <row r="66" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A66" s="4"/>
+      <c r="A66" s="7"/>
       <c r="B66" s="7"/>
       <c r="C66" s="7"/>
       <c r="D66" s="11"/>
@@ -28349,46 +28312,18 @@
       <c r="Y991" s="7"/>
       <c r="Z991" s="7"/>
     </row>
-    <row r="992" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A992" s="7"/>
-      <c r="B992" s="7"/>
-      <c r="C992" s="7"/>
-      <c r="D992" s="11"/>
-      <c r="E992" s="7"/>
-      <c r="F992" s="12"/>
-      <c r="G992" s="12"/>
-      <c r="H992" s="12"/>
-      <c r="I992" s="11"/>
-      <c r="J992" s="12"/>
-      <c r="K992" s="11"/>
-      <c r="L992" s="12"/>
-      <c r="M992" s="12"/>
-      <c r="N992" s="7"/>
-      <c r="O992" s="7"/>
-      <c r="P992" s="7"/>
-      <c r="Q992" s="7"/>
-      <c r="R992" s="7"/>
-      <c r="S992" s="7"/>
-      <c r="T992" s="7"/>
-      <c r="U992" s="7"/>
-      <c r="V992" s="7"/>
-      <c r="W992" s="7"/>
-      <c r="X992" s="7"/>
-      <c r="Y992" s="7"/>
-      <c r="Z992" s="7"/>
-    </row>
   </sheetData>
   <dataValidations count="4">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C49:C992 C25:C37 C1:C23" xr:uid="{00000000-0002-0000-0000-000002000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C48:C991 C24:C36 C1:C22" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>"nominal,ordinal,interval,ratio,dateTime"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E25:E992 E1:E23" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E24:E991 E1:E22" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"text,enumerated,dateTime,numeric"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F25:F992 F1:F23" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F24:F991 F1:F22" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"ratio,interval"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H25:H992 H1:H23" xr:uid="{00000000-0002-0000-0000-000003000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H24:H991 H1:H22" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>"natural,whole,integer,real"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
cleans name on redd sumary table and metadata
</commit_message>
<xml_diff>
--- a/data-raw/metadata/clear_redd_summary_metadata.xlsx
+++ b/data-raw/metadata/clear_redd_summary_metadata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Badhia\Documents\git\jpe-clear-adult-edi\data-raw\metadata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B91AFB5-A8EA-42CE-8437-5945C64FE1A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C808BF5A-C54F-47B7-A531-689225053B97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5650" yWindow="2160" windowWidth="19200" windowHeight="11170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -136,10 +136,10 @@
     <t>7</t>
   </si>
   <si>
-    <t>reaches_numbers</t>
+    <t>Survey reach(es) where survey was done</t>
   </si>
   <si>
-    <t>Survey reach(es) where survey was done</t>
+    <t>reach_numbers</t>
   </si>
 </sst>
 </file>
@@ -682,10 +682,10 @@
     </row>
     <row r="5" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>31</v>

</xml_diff>